<commit_message>
Updated analysis scripts and cleaned code
</commit_message>
<xml_diff>
--- a/manu_sourcedata/suppl_tables.xlsx
+++ b/manu_sourcedata/suppl_tables.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manu_sourcedata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1760A00E-6C24-9444-9F7B-753BC8E72E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF08C09-08EE-EC46-85AE-1E05DC5F7854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38120" yWindow="7040" windowWidth="27640" windowHeight="16940" activeTab="2" xr2:uid="{07063887-18E2-9747-8ACB-521C19DAFDA2}"/>
+    <workbookView xWindow="48320" yWindow="2540" windowWidth="34560" windowHeight="21580" activeTab="4" xr2:uid="{07063887-18E2-9747-8ACB-521C19DAFDA2}"/>
   </bookViews>
   <sheets>
     <sheet name="1 xenium panel" sheetId="1" r:id="rId1"/>
     <sheet name="2 ind T cell subtype prop" sheetId="2" r:id="rId2"/>
     <sheet name="3 ind B cell subtype prop" sheetId="3" r:id="rId3"/>
+    <sheet name="4 TCR probes and samples" sheetId="4" r:id="rId4"/>
+    <sheet name="5 filtered gene lists" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="525">
   <si>
     <t>CDH19</t>
   </si>
@@ -1544,19 +1546,465 @@
   </si>
   <si>
     <t>PBBKFP_PT</t>
+  </si>
+  <si>
+    <t>Sequence</t>
+  </si>
+  <si>
+    <r>
+      <t>clone58_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLGYEQYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone68_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSFLSSYNEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone69_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSPGTSGTDTQYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone71_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLLGAGNTIYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone72_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLIGAGNTIYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone73_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLAGQETQYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone74_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLVASGGYNEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone78_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASTSSSYNEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone86_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSPGLALYEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone88_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLIGTYNEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone90_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSQDLVEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone91_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSPDRTYEQYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone93_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSPEGDTQYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone94_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSPQGDTIYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone96_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLPDTGELFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone97_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSETSGRADEQFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone98_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSSGTSGMDTQYF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>clone100_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>CASSLTGNTEAFF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_TRB</t>
+    </r>
+  </si>
+  <si>
+    <t>Caushi</t>
+  </si>
+  <si>
+    <t>Oliveira</t>
+  </si>
+  <si>
+    <t>Lowery</t>
+  </si>
+  <si>
+    <t>Hanada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1579,8 +2027,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4876,4 +5339,2072 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B48EF9-98EE-9446-B8E9-8DACAA829D87}">
+  <dimension ref="A1:K100"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5">
+        <v>1</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5">
+        <v>1</v>
+      </c>
+      <c r="K6" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B7" s="5">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5">
+        <v>1</v>
+      </c>
+      <c r="K7" s="5"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4">
+        <v>1</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5">
+        <v>1</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1</v>
+      </c>
+      <c r="J12" s="5">
+        <v>1</v>
+      </c>
+      <c r="K12" s="5"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B15" s="5">
+        <v>1</v>
+      </c>
+      <c r="C15" s="5">
+        <v>1</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5">
+        <v>1</v>
+      </c>
+      <c r="I16" s="5">
+        <v>1</v>
+      </c>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5">
+        <v>1</v>
+      </c>
+      <c r="H17" s="5">
+        <v>1</v>
+      </c>
+      <c r="I17" s="5">
+        <v>1</v>
+      </c>
+      <c r="J17" s="5">
+        <v>1</v>
+      </c>
+      <c r="K17" s="5"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5">
+        <v>1</v>
+      </c>
+      <c r="E18" s="5">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5">
+        <v>1</v>
+      </c>
+      <c r="H18" s="5">
+        <v>1</v>
+      </c>
+      <c r="I18" s="5">
+        <v>1</v>
+      </c>
+      <c r="J18" s="5">
+        <v>1</v>
+      </c>
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B19" s="5">
+        <v>1</v>
+      </c>
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5">
+        <v>1</v>
+      </c>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5">
+        <v>1</v>
+      </c>
+      <c r="K19" s="5"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5">
+        <v>1</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5">
+        <v>1</v>
+      </c>
+      <c r="H20" s="5">
+        <v>1</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5">
+        <v>1</v>
+      </c>
+      <c r="K20" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5">
+        <v>1</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5">
+        <v>1</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B23" s="5">
+        <v>1</v>
+      </c>
+      <c r="C23" s="5">
+        <v>1</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B24" s="5">
+        <v>1</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5">
+        <v>1</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5">
+        <v>1</v>
+      </c>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5">
+        <v>1</v>
+      </c>
+      <c r="E27" s="5">
+        <v>1</v>
+      </c>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5">
+        <v>1</v>
+      </c>
+      <c r="G28" s="5">
+        <v>1</v>
+      </c>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="B29" s="4">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4">
+        <v>1</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5">
+        <v>1</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5">
+        <v>1</v>
+      </c>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5">
+        <v>1</v>
+      </c>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="B34" s="5">
+        <v>1</v>
+      </c>
+      <c r="C34" s="5">
+        <v>1</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5">
+        <v>1</v>
+      </c>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B36" s="5">
+        <v>1</v>
+      </c>
+      <c r="C36" s="5">
+        <v>1</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B37" s="5">
+        <v>1</v>
+      </c>
+      <c r="C37" s="5">
+        <v>1</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5">
+        <v>1</v>
+      </c>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5">
+        <v>1</v>
+      </c>
+      <c r="I38" s="5">
+        <v>1</v>
+      </c>
+      <c r="J38" s="5">
+        <v>1</v>
+      </c>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5">
+        <v>1</v>
+      </c>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5">
+        <v>1</v>
+      </c>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5">
+        <v>1</v>
+      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5">
+        <v>1</v>
+      </c>
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5">
+        <v>1</v>
+      </c>
+      <c r="D40" s="5">
+        <v>1</v>
+      </c>
+      <c r="E40" s="5">
+        <v>1</v>
+      </c>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5">
+        <v>1</v>
+      </c>
+      <c r="K40" s="5"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5">
+        <v>1</v>
+      </c>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5">
+        <v>1</v>
+      </c>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5">
+        <v>1</v>
+      </c>
+      <c r="K41" s="5"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5">
+        <v>1</v>
+      </c>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5">
+        <v>1</v>
+      </c>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5">
+        <v>1</v>
+      </c>
+      <c r="K42" s="5"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5">
+        <v>1</v>
+      </c>
+      <c r="D43" s="5">
+        <v>1</v>
+      </c>
+      <c r="E43" s="5">
+        <v>1</v>
+      </c>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5">
+        <v>1</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5">
+        <v>1</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="B46" s="4">
+        <v>1</v>
+      </c>
+      <c r="C46" s="4">
+        <v>1</v>
+      </c>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5">
+        <v>1</v>
+      </c>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5">
+        <v>1</v>
+      </c>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5">
+        <v>1</v>
+      </c>
+      <c r="K47" s="5"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5">
+        <v>1</v>
+      </c>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5">
+        <v>1</v>
+      </c>
+      <c r="G49" s="5">
+        <v>1</v>
+      </c>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4">
+        <v>1</v>
+      </c>
+      <c r="E50" s="4">
+        <v>1</v>
+      </c>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5">
+        <v>1</v>
+      </c>
+      <c r="I51" s="5">
+        <v>1</v>
+      </c>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A52" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="B52" s="4">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4">
+        <v>1</v>
+      </c>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="B53" s="4">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4">
+        <v>1</v>
+      </c>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5"/>
+      <c r="D54" s="5">
+        <v>1</v>
+      </c>
+      <c r="E54" s="5">
+        <v>1</v>
+      </c>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5">
+        <v>1</v>
+      </c>
+      <c r="K55" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5">
+        <v>1</v>
+      </c>
+      <c r="K56" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="B57" s="4">
+        <v>1</v>
+      </c>
+      <c r="C57" s="4">
+        <v>1</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4">
+        <v>1</v>
+      </c>
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5">
+        <v>1</v>
+      </c>
+      <c r="I58" s="5"/>
+      <c r="J58" s="5">
+        <v>1</v>
+      </c>
+      <c r="K58" s="5"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5">
+        <v>1</v>
+      </c>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5">
+        <v>1</v>
+      </c>
+      <c r="J59" s="5"/>
+      <c r="K59" s="5"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="B60" s="4">
+        <v>1</v>
+      </c>
+      <c r="C60" s="4">
+        <v>1</v>
+      </c>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5">
+        <v>1</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5">
+        <v>1</v>
+      </c>
+      <c r="K61" s="5"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B62" s="4">
+        <v>1</v>
+      </c>
+      <c r="C62" s="4">
+        <v>1</v>
+      </c>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5">
+        <v>1</v>
+      </c>
+      <c r="E63" s="5">
+        <v>1</v>
+      </c>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="K63" s="5"/>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B64" s="4">
+        <v>1</v>
+      </c>
+      <c r="C64" s="4">
+        <v>1</v>
+      </c>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4">
+        <v>1</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4"/>
+      <c r="J65" s="4"/>
+      <c r="K65" s="4"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5">
+        <v>1</v>
+      </c>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="5"/>
+      <c r="K66" s="5"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5">
+        <v>1</v>
+      </c>
+      <c r="K67" s="5"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5">
+        <v>1</v>
+      </c>
+      <c r="I68" s="5"/>
+      <c r="J68" s="5"/>
+      <c r="K68" s="5"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="5">
+        <v>1</v>
+      </c>
+      <c r="K69" s="5"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5">
+        <v>1</v>
+      </c>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="5"/>
+      <c r="K70" s="5"/>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5">
+        <v>1</v>
+      </c>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="K71" s="5"/>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="B72" s="5"/>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5">
+        <v>1</v>
+      </c>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="K72" s="5"/>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="B73" s="5"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="5"/>
+      <c r="H73" s="5"/>
+      <c r="I73" s="5"/>
+      <c r="J73" s="5">
+        <v>1</v>
+      </c>
+      <c r="K73" s="5"/>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="B74" s="5"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5">
+        <v>1</v>
+      </c>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5"/>
+      <c r="I74" s="5"/>
+      <c r="J74" s="5"/>
+      <c r="K74" s="5"/>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B75" s="5"/>
+      <c r="C75" s="5"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="5">
+        <v>1</v>
+      </c>
+      <c r="I75" s="5"/>
+      <c r="J75" s="5"/>
+      <c r="K75" s="5"/>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="5">
+        <v>1</v>
+      </c>
+      <c r="I76" s="5"/>
+      <c r="J76" s="5"/>
+      <c r="K76" s="5"/>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5">
+        <v>1</v>
+      </c>
+      <c r="H77" s="5"/>
+      <c r="I77" s="5"/>
+      <c r="J77" s="5"/>
+      <c r="K77" s="5"/>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="B78" s="5"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5">
+        <v>1</v>
+      </c>
+      <c r="H78" s="5"/>
+      <c r="I78" s="5"/>
+      <c r="J78" s="5"/>
+      <c r="K78" s="5"/>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B79" s="5"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="5">
+        <v>1</v>
+      </c>
+      <c r="I79" s="5"/>
+      <c r="J79" s="5"/>
+      <c r="K79" s="5"/>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B80" s="5"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+      <c r="H80" s="5"/>
+      <c r="I80" s="5">
+        <v>1</v>
+      </c>
+      <c r="J80" s="5"/>
+      <c r="K80" s="5"/>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B81" s="5"/>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5"/>
+      <c r="I81" s="5"/>
+      <c r="J81" s="5">
+        <v>1</v>
+      </c>
+      <c r="K81" s="5"/>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="B82" s="5"/>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5"/>
+      <c r="I82" s="5"/>
+      <c r="J82" s="5"/>
+      <c r="K82" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B83" s="5"/>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5">
+        <v>1</v>
+      </c>
+      <c r="I83" s="5">
+        <v>1</v>
+      </c>
+      <c r="J83" s="5"/>
+      <c r="K83" s="5"/>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B84" s="5">
+        <v>1</v>
+      </c>
+      <c r="C84" s="5">
+        <v>1</v>
+      </c>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5"/>
+      <c r="I84" s="5"/>
+      <c r="J84" s="5"/>
+      <c r="K84" s="5"/>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B85" s="5"/>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5">
+        <v>1</v>
+      </c>
+      <c r="E85" s="5">
+        <v>1</v>
+      </c>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="5"/>
+      <c r="J85" s="5"/>
+      <c r="K85" s="5"/>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B86" s="5"/>
+      <c r="C86" s="5"/>
+      <c r="D86" s="5">
+        <v>1</v>
+      </c>
+      <c r="E86" s="5">
+        <v>1</v>
+      </c>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5"/>
+      <c r="H86" s="5"/>
+      <c r="I86" s="5"/>
+      <c r="J86" s="5"/>
+      <c r="K86" s="5"/>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="B87" s="4">
+        <v>1</v>
+      </c>
+      <c r="C87" s="4">
+        <v>1</v>
+      </c>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
+      <c r="G87" s="4"/>
+      <c r="H87" s="4"/>
+      <c r="I87" s="4"/>
+      <c r="J87" s="4"/>
+      <c r="K87" s="4"/>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="B88" s="5"/>
+      <c r="C88" s="5"/>
+      <c r="D88" s="5">
+        <v>1</v>
+      </c>
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5"/>
+      <c r="H88" s="5"/>
+      <c r="I88" s="5"/>
+      <c r="J88" s="5"/>
+      <c r="K88" s="5"/>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5">
+        <v>1</v>
+      </c>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="5"/>
+      <c r="J89" s="5"/>
+      <c r="K89" s="5"/>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5">
+        <v>1</v>
+      </c>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="5"/>
+      <c r="K90" s="5"/>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="B91" s="5"/>
+      <c r="C91" s="5"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5"/>
+      <c r="I91" s="5"/>
+      <c r="J91" s="5">
+        <v>1</v>
+      </c>
+      <c r="K91" s="5"/>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B92" s="5"/>
+      <c r="C92" s="5"/>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5">
+        <v>1</v>
+      </c>
+      <c r="I92" s="5"/>
+      <c r="J92" s="5"/>
+      <c r="K92" s="5"/>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B93" s="5"/>
+      <c r="C93" s="5"/>
+      <c r="D93" s="5"/>
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5">
+        <v>1</v>
+      </c>
+      <c r="I93" s="5"/>
+      <c r="J93" s="5"/>
+      <c r="K93" s="5"/>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="B94" s="5"/>
+      <c r="C94" s="5"/>
+      <c r="D94" s="5"/>
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+      <c r="I94" s="5"/>
+      <c r="J94" s="5">
+        <v>1</v>
+      </c>
+      <c r="K94" s="5"/>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B95" s="5">
+        <v>1</v>
+      </c>
+      <c r="C95" s="5">
+        <v>1</v>
+      </c>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+      <c r="I95" s="5"/>
+      <c r="J95" s="5"/>
+      <c r="K95" s="5"/>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="B96" s="5"/>
+      <c r="C96" s="5"/>
+      <c r="D96" s="5"/>
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5"/>
+      <c r="H96" s="5">
+        <v>1</v>
+      </c>
+      <c r="I96" s="5"/>
+      <c r="J96" s="5"/>
+      <c r="K96" s="5"/>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="B97" s="5"/>
+      <c r="C97" s="5"/>
+      <c r="D97" s="5">
+        <v>1</v>
+      </c>
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="5"/>
+      <c r="I97" s="5"/>
+      <c r="J97" s="5"/>
+      <c r="K97" s="5"/>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+      <c r="H98" s="5"/>
+      <c r="I98" s="5"/>
+      <c r="J98" s="5">
+        <v>1</v>
+      </c>
+      <c r="K98" s="5"/>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B99" s="5"/>
+      <c r="C99" s="5"/>
+      <c r="D99" s="5"/>
+      <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="5">
+        <v>1</v>
+      </c>
+      <c r="I99" s="5"/>
+      <c r="J99" s="5"/>
+      <c r="K99" s="5"/>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="B100" s="5"/>
+      <c r="C100" s="5"/>
+      <c r="D100" s="5"/>
+      <c r="E100" s="5"/>
+      <c r="F100" s="5"/>
+      <c r="G100" s="5">
+        <v>1</v>
+      </c>
+      <c r="H100" s="5"/>
+      <c r="I100" s="5"/>
+      <c r="J100" s="5"/>
+      <c r="K100" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{099D8DB7-1C01-8040-BBF1-2F2FE6508470}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B1" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1" t="s">
+        <v>523</v>
+      </c>
+      <c r="D1" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>349</v>
+      </c>
+      <c r="D2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>358</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Edited manuscript and corresponding figures for better flow
</commit_message>
<xml_diff>
--- a/manu_sourcedata/suppl_tables.xlsx
+++ b/manu_sourcedata/suppl_tables.xlsx
@@ -8,17 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manu_sourcedata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695E4CFA-A563-A54D-8F52-8D70188FFC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089507A9-F083-734B-BEC0-A43340A448B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48320" yWindow="2540" windowWidth="34560" windowHeight="21580" activeTab="3" xr2:uid="{07063887-18E2-9747-8ACB-521C19DAFDA2}"/>
+    <workbookView xWindow="-7900" yWindow="-28300" windowWidth="33680" windowHeight="12580" activeTab="2" xr2:uid="{07063887-18E2-9747-8ACB-521C19DAFDA2}"/>
   </bookViews>
   <sheets>
-    <sheet name="1 xenium panel" sheetId="1" r:id="rId1"/>
-    <sheet name="2 ind T cell subtype prop" sheetId="2" r:id="rId2"/>
-    <sheet name="3a ind B cell subtype prop" sheetId="3" r:id="rId3"/>
-    <sheet name="3b ind B cell subtype prop stat" sheetId="6" r:id="rId4"/>
-    <sheet name="4 TCR probes and samples" sheetId="4" r:id="rId5"/>
-    <sheet name="5 filtered gene lists" sheetId="5" r:id="rId6"/>
+    <sheet name="1 TCR probes and samples" sheetId="4" r:id="rId1"/>
+    <sheet name="2 xenium panel" sheetId="1" r:id="rId2"/>
+    <sheet name="3 ind T cell subtype prop" sheetId="2" r:id="rId3"/>
+    <sheet name="4 filtered gene lists" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="519">
   <si>
     <t>CDH19</t>
   </si>
@@ -1492,31 +1490,7 @@
     <t>gdT</t>
   </si>
   <si>
-    <t>Activated B</t>
-  </si>
-  <si>
-    <t>Naive B</t>
-  </si>
-  <si>
-    <t>Plasma</t>
-  </si>
-  <si>
-    <t>Proliferating memory B</t>
-  </si>
-  <si>
-    <t>cDC</t>
-  </si>
-  <si>
-    <t>pDC</t>
-  </si>
-  <si>
     <t>sample</t>
-  </si>
-  <si>
-    <t>Cytotoxic CD8T</t>
-  </si>
-  <si>
-    <t>Proliferating CD8T</t>
   </si>
   <si>
     <t>PAZNRG_DX</t>
@@ -1978,37 +1952,10 @@
     <t>Hanada</t>
   </si>
   <si>
-    <t>T_subtype</t>
-  </si>
-  <si>
-    <t>n_pairs</t>
-  </si>
-  <si>
-    <t>mean_DX</t>
-  </si>
-  <si>
-    <t>mean_PT</t>
-  </si>
-  <si>
-    <t>mean_delta_PT_minus_DX</t>
-  </si>
-  <si>
-    <t>median_DX</t>
-  </si>
-  <si>
-    <t>median_PT</t>
-  </si>
-  <si>
-    <t>median_delta_PT_minus_DX</t>
-  </si>
-  <si>
-    <t>wilcoxon_stat</t>
-  </si>
-  <si>
-    <t>p_value</t>
-  </si>
-  <si>
-    <t>p_value_fdr</t>
+    <t>Cytotoxic T</t>
+  </si>
+  <si>
+    <t>Proliferating T</t>
   </si>
 </sst>
 </file>
@@ -2411,6 +2358,1921 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B48EF9-98EE-9446-B8E9-8DACAA829D87}">
+  <dimension ref="A1:K100"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5">
+        <v>1</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5">
+        <v>1</v>
+      </c>
+      <c r="K6" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B7" s="5">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5">
+        <v>1</v>
+      </c>
+      <c r="K7" s="5"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4">
+        <v>1</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5">
+        <v>1</v>
+      </c>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5">
+        <v>1</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1</v>
+      </c>
+      <c r="J12" s="5">
+        <v>1</v>
+      </c>
+      <c r="K12" s="5"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B15" s="5">
+        <v>1</v>
+      </c>
+      <c r="C15" s="5">
+        <v>1</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5">
+        <v>1</v>
+      </c>
+      <c r="I16" s="5">
+        <v>1</v>
+      </c>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5">
+        <v>1</v>
+      </c>
+      <c r="H17" s="5">
+        <v>1</v>
+      </c>
+      <c r="I17" s="5">
+        <v>1</v>
+      </c>
+      <c r="J17" s="5">
+        <v>1</v>
+      </c>
+      <c r="K17" s="5"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5">
+        <v>1</v>
+      </c>
+      <c r="E18" s="5">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5">
+        <v>1</v>
+      </c>
+      <c r="H18" s="5">
+        <v>1</v>
+      </c>
+      <c r="I18" s="5">
+        <v>1</v>
+      </c>
+      <c r="J18" s="5">
+        <v>1</v>
+      </c>
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B19" s="5">
+        <v>1</v>
+      </c>
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5">
+        <v>1</v>
+      </c>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5">
+        <v>1</v>
+      </c>
+      <c r="K19" s="5"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5">
+        <v>1</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5">
+        <v>1</v>
+      </c>
+      <c r="H20" s="5">
+        <v>1</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5">
+        <v>1</v>
+      </c>
+      <c r="K20" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5">
+        <v>1</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5">
+        <v>1</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B23" s="5">
+        <v>1</v>
+      </c>
+      <c r="C23" s="5">
+        <v>1</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B24" s="5">
+        <v>1</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5">
+        <v>1</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5">
+        <v>1</v>
+      </c>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5">
+        <v>1</v>
+      </c>
+      <c r="E27" s="5">
+        <v>1</v>
+      </c>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5">
+        <v>1</v>
+      </c>
+      <c r="G28" s="5">
+        <v>1</v>
+      </c>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="B29" s="4">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4">
+        <v>1</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5">
+        <v>1</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5">
+        <v>1</v>
+      </c>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5">
+        <v>1</v>
+      </c>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="B34" s="5">
+        <v>1</v>
+      </c>
+      <c r="C34" s="5">
+        <v>1</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5">
+        <v>1</v>
+      </c>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B36" s="5">
+        <v>1</v>
+      </c>
+      <c r="C36" s="5">
+        <v>1</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B37" s="5">
+        <v>1</v>
+      </c>
+      <c r="C37" s="5">
+        <v>1</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5">
+        <v>1</v>
+      </c>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5">
+        <v>1</v>
+      </c>
+      <c r="I38" s="5">
+        <v>1</v>
+      </c>
+      <c r="J38" s="5">
+        <v>1</v>
+      </c>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5">
+        <v>1</v>
+      </c>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5">
+        <v>1</v>
+      </c>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5">
+        <v>1</v>
+      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5">
+        <v>1</v>
+      </c>
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5">
+        <v>1</v>
+      </c>
+      <c r="D40" s="5">
+        <v>1</v>
+      </c>
+      <c r="E40" s="5">
+        <v>1</v>
+      </c>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5">
+        <v>1</v>
+      </c>
+      <c r="K40" s="5"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5">
+        <v>1</v>
+      </c>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5">
+        <v>1</v>
+      </c>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5">
+        <v>1</v>
+      </c>
+      <c r="K41" s="5"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5">
+        <v>1</v>
+      </c>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5">
+        <v>1</v>
+      </c>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5">
+        <v>1</v>
+      </c>
+      <c r="K42" s="5"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5">
+        <v>1</v>
+      </c>
+      <c r="D43" s="5">
+        <v>1</v>
+      </c>
+      <c r="E43" s="5">
+        <v>1</v>
+      </c>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5">
+        <v>1</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5">
+        <v>1</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="B46" s="4">
+        <v>1</v>
+      </c>
+      <c r="C46" s="4">
+        <v>1</v>
+      </c>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5">
+        <v>1</v>
+      </c>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5">
+        <v>1</v>
+      </c>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5">
+        <v>1</v>
+      </c>
+      <c r="K47" s="5"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5">
+        <v>1</v>
+      </c>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5">
+        <v>1</v>
+      </c>
+      <c r="G49" s="5">
+        <v>1</v>
+      </c>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4">
+        <v>1</v>
+      </c>
+      <c r="E50" s="4">
+        <v>1</v>
+      </c>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5">
+        <v>1</v>
+      </c>
+      <c r="I51" s="5">
+        <v>1</v>
+      </c>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A52" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="B52" s="4">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4">
+        <v>1</v>
+      </c>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="B53" s="4">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4">
+        <v>1</v>
+      </c>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+      <c r="H53" s="4"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="4"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5"/>
+      <c r="D54" s="5">
+        <v>1</v>
+      </c>
+      <c r="E54" s="5">
+        <v>1</v>
+      </c>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5">
+        <v>1</v>
+      </c>
+      <c r="K55" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5">
+        <v>1</v>
+      </c>
+      <c r="K56" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="B57" s="4">
+        <v>1</v>
+      </c>
+      <c r="C57" s="4">
+        <v>1</v>
+      </c>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4">
+        <v>1</v>
+      </c>
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="B58" s="5"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5">
+        <v>1</v>
+      </c>
+      <c r="I58" s="5"/>
+      <c r="J58" s="5">
+        <v>1</v>
+      </c>
+      <c r="K58" s="5"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B59" s="5"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5">
+        <v>1</v>
+      </c>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5">
+        <v>1</v>
+      </c>
+      <c r="J59" s="5"/>
+      <c r="K59" s="5"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="B60" s="4">
+        <v>1</v>
+      </c>
+      <c r="C60" s="4">
+        <v>1</v>
+      </c>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5">
+        <v>1</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5">
+        <v>1</v>
+      </c>
+      <c r="K61" s="5"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B62" s="4">
+        <v>1</v>
+      </c>
+      <c r="C62" s="4">
+        <v>1</v>
+      </c>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5">
+        <v>1</v>
+      </c>
+      <c r="E63" s="5">
+        <v>1</v>
+      </c>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="K63" s="5"/>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B64" s="4">
+        <v>1</v>
+      </c>
+      <c r="C64" s="4">
+        <v>1</v>
+      </c>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4">
+        <v>1</v>
+      </c>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+      <c r="H65" s="4"/>
+      <c r="I65" s="4"/>
+      <c r="J65" s="4"/>
+      <c r="K65" s="4"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B66" s="5"/>
+      <c r="C66" s="5">
+        <v>1</v>
+      </c>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="5"/>
+      <c r="K66" s="5"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5">
+        <v>1</v>
+      </c>
+      <c r="K67" s="5"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5">
+        <v>1</v>
+      </c>
+      <c r="I68" s="5"/>
+      <c r="J68" s="5"/>
+      <c r="K68" s="5"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="5">
+        <v>1</v>
+      </c>
+      <c r="K69" s="5"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5">
+        <v>1</v>
+      </c>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="5"/>
+      <c r="K70" s="5"/>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5">
+        <v>1</v>
+      </c>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="K71" s="5"/>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="B72" s="5"/>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5">
+        <v>1</v>
+      </c>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="K72" s="5"/>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B73" s="5"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="5"/>
+      <c r="H73" s="5"/>
+      <c r="I73" s="5"/>
+      <c r="J73" s="5">
+        <v>1</v>
+      </c>
+      <c r="K73" s="5"/>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="B74" s="5"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5">
+        <v>1</v>
+      </c>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5"/>
+      <c r="I74" s="5"/>
+      <c r="J74" s="5"/>
+      <c r="K74" s="5"/>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B75" s="5"/>
+      <c r="C75" s="5"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5"/>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="5">
+        <v>1</v>
+      </c>
+      <c r="I75" s="5"/>
+      <c r="J75" s="5"/>
+      <c r="K75" s="5"/>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="5">
+        <v>1</v>
+      </c>
+      <c r="I76" s="5"/>
+      <c r="J76" s="5"/>
+      <c r="K76" s="5"/>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5">
+        <v>1</v>
+      </c>
+      <c r="H77" s="5"/>
+      <c r="I77" s="5"/>
+      <c r="J77" s="5"/>
+      <c r="K77" s="5"/>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B78" s="5"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="5">
+        <v>1</v>
+      </c>
+      <c r="H78" s="5"/>
+      <c r="I78" s="5"/>
+      <c r="J78" s="5"/>
+      <c r="K78" s="5"/>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B79" s="5"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="5"/>
+      <c r="H79" s="5">
+        <v>1</v>
+      </c>
+      <c r="I79" s="5"/>
+      <c r="J79" s="5"/>
+      <c r="K79" s="5"/>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B80" s="5"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
+      <c r="H80" s="5"/>
+      <c r="I80" s="5">
+        <v>1</v>
+      </c>
+      <c r="J80" s="5"/>
+      <c r="K80" s="5"/>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B81" s="5"/>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5"/>
+      <c r="I81" s="5"/>
+      <c r="J81" s="5">
+        <v>1</v>
+      </c>
+      <c r="K81" s="5"/>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="B82" s="5"/>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5"/>
+      <c r="I82" s="5"/>
+      <c r="J82" s="5"/>
+      <c r="K82" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B83" s="5"/>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5">
+        <v>1</v>
+      </c>
+      <c r="I83" s="5">
+        <v>1</v>
+      </c>
+      <c r="J83" s="5"/>
+      <c r="K83" s="5"/>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B84" s="5">
+        <v>1</v>
+      </c>
+      <c r="C84" s="5">
+        <v>1</v>
+      </c>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="5"/>
+      <c r="G84" s="5"/>
+      <c r="H84" s="5"/>
+      <c r="I84" s="5"/>
+      <c r="J84" s="5"/>
+      <c r="K84" s="5"/>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B85" s="5"/>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5">
+        <v>1</v>
+      </c>
+      <c r="E85" s="5">
+        <v>1</v>
+      </c>
+      <c r="F85" s="5"/>
+      <c r="G85" s="5"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="5"/>
+      <c r="J85" s="5"/>
+      <c r="K85" s="5"/>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="B86" s="5"/>
+      <c r="C86" s="5"/>
+      <c r="D86" s="5">
+        <v>1</v>
+      </c>
+      <c r="E86" s="5">
+        <v>1</v>
+      </c>
+      <c r="F86" s="5"/>
+      <c r="G86" s="5"/>
+      <c r="H86" s="5"/>
+      <c r="I86" s="5"/>
+      <c r="J86" s="5"/>
+      <c r="K86" s="5"/>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="B87" s="4">
+        <v>1</v>
+      </c>
+      <c r="C87" s="4">
+        <v>1</v>
+      </c>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
+      <c r="G87" s="4"/>
+      <c r="H87" s="4"/>
+      <c r="I87" s="4"/>
+      <c r="J87" s="4"/>
+      <c r="K87" s="4"/>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="B88" s="5"/>
+      <c r="C88" s="5"/>
+      <c r="D88" s="5">
+        <v>1</v>
+      </c>
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
+      <c r="G88" s="5"/>
+      <c r="H88" s="5"/>
+      <c r="I88" s="5"/>
+      <c r="J88" s="5"/>
+      <c r="K88" s="5"/>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5">
+        <v>1</v>
+      </c>
+      <c r="F89" s="5"/>
+      <c r="G89" s="5"/>
+      <c r="H89" s="5"/>
+      <c r="I89" s="5"/>
+      <c r="J89" s="5"/>
+      <c r="K89" s="5"/>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5">
+        <v>1</v>
+      </c>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="5"/>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5"/>
+      <c r="J90" s="5"/>
+      <c r="K90" s="5"/>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="B91" s="5"/>
+      <c r="C91" s="5"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+      <c r="F91" s="5"/>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5"/>
+      <c r="I91" s="5"/>
+      <c r="J91" s="5">
+        <v>1</v>
+      </c>
+      <c r="K91" s="5"/>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B92" s="5"/>
+      <c r="C92" s="5"/>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5">
+        <v>1</v>
+      </c>
+      <c r="I92" s="5"/>
+      <c r="J92" s="5"/>
+      <c r="K92" s="5"/>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="B93" s="5"/>
+      <c r="C93" s="5"/>
+      <c r="D93" s="5"/>
+      <c r="E93" s="5"/>
+      <c r="F93" s="5"/>
+      <c r="G93" s="5"/>
+      <c r="H93" s="5">
+        <v>1</v>
+      </c>
+      <c r="I93" s="5"/>
+      <c r="J93" s="5"/>
+      <c r="K93" s="5"/>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="B94" s="5"/>
+      <c r="C94" s="5"/>
+      <c r="D94" s="5"/>
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
+      <c r="I94" s="5"/>
+      <c r="J94" s="5">
+        <v>1</v>
+      </c>
+      <c r="K94" s="5"/>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B95" s="5">
+        <v>1</v>
+      </c>
+      <c r="C95" s="5">
+        <v>1</v>
+      </c>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+      <c r="I95" s="5"/>
+      <c r="J95" s="5"/>
+      <c r="K95" s="5"/>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="B96" s="5"/>
+      <c r="C96" s="5"/>
+      <c r="D96" s="5"/>
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5"/>
+      <c r="H96" s="5">
+        <v>1</v>
+      </c>
+      <c r="I96" s="5"/>
+      <c r="J96" s="5"/>
+      <c r="K96" s="5"/>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="B97" s="5"/>
+      <c r="C97" s="5"/>
+      <c r="D97" s="5">
+        <v>1</v>
+      </c>
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="5"/>
+      <c r="I97" s="5"/>
+      <c r="J97" s="5"/>
+      <c r="K97" s="5"/>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+      <c r="H98" s="5"/>
+      <c r="I98" s="5"/>
+      <c r="J98" s="5">
+        <v>1</v>
+      </c>
+      <c r="K98" s="5"/>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B99" s="5"/>
+      <c r="C99" s="5"/>
+      <c r="D99" s="5"/>
+      <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
+      <c r="H99" s="5">
+        <v>1</v>
+      </c>
+      <c r="I99" s="5"/>
+      <c r="J99" s="5"/>
+      <c r="K99" s="5"/>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="B100" s="5"/>
+      <c r="C100" s="5"/>
+      <c r="D100" s="5"/>
+      <c r="E100" s="5"/>
+      <c r="F100" s="5"/>
+      <c r="G100" s="5">
+        <v>1</v>
+      </c>
+      <c r="H100" s="5"/>
+      <c r="I100" s="5"/>
+      <c r="J100" s="5"/>
+      <c r="K100" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67ADC079-0F11-4146-BE13-534595A0699B}">
   <dimension ref="A1:A477"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4808,7 +6670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32B9795E-0DC1-AF41-BB10-8912F9FB10D9}">
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4820,19 +6682,19 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="B1" t="s">
         <v>477</v>
       </c>
       <c r="C1" t="s">
-        <v>490</v>
+        <v>517</v>
       </c>
       <c r="D1" t="s">
         <v>479</v>
       </c>
       <c r="E1" t="s">
-        <v>491</v>
+        <v>518</v>
       </c>
       <c r="F1" t="s">
         <v>480</v>
@@ -4843,7 +6705,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
       <c r="B2" t="s">
         <v>478</v>
@@ -4866,7 +6728,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="B3" t="s">
         <v>481</v>
@@ -4889,7 +6751,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="B4" t="s">
         <v>478</v>
@@ -4912,7 +6774,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="B5" t="s">
         <v>481</v>
@@ -4935,7 +6797,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="B6" t="s">
         <v>478</v>
@@ -4958,7 +6820,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="B7" t="s">
         <v>481</v>
@@ -4981,7 +6843,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="B8" t="s">
         <v>478</v>
@@ -5004,7 +6866,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
       <c r="B9" t="s">
         <v>481</v>
@@ -5027,7 +6889,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="B10" t="s">
         <v>478</v>
@@ -5050,7 +6912,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="B11" t="s">
         <v>481</v>
@@ -5069,305 +6931,6 @@
       </c>
       <c r="G11">
         <v>3.3592789840229398E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58735501-D637-E444-B193-7DB34582E683}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="20.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>489</v>
-      </c>
-      <c r="B1" t="s">
-        <v>477</v>
-      </c>
-      <c r="C1" t="s">
-        <v>483</v>
-      </c>
-      <c r="D1" t="s">
-        <v>484</v>
-      </c>
-      <c r="E1" t="s">
-        <v>485</v>
-      </c>
-      <c r="F1" t="s">
-        <v>486</v>
-      </c>
-      <c r="G1" t="s">
-        <v>487</v>
-      </c>
-      <c r="H1" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>492</v>
-      </c>
-      <c r="B2" t="s">
-        <v>478</v>
-      </c>
-      <c r="C2">
-        <v>4.8786022237349604E-3</v>
-      </c>
-      <c r="D2">
-        <v>0.95121397776265004</v>
-      </c>
-      <c r="E2">
-        <v>5.1055139550714697E-3</v>
-      </c>
-      <c r="F2">
-        <v>8.2822781937826103E-3</v>
-      </c>
-      <c r="G2">
-        <v>2.0989335148627102E-2</v>
-      </c>
-      <c r="H2">
-        <v>9.5302927161334192E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>493</v>
-      </c>
-      <c r="B3" t="s">
-        <v>481</v>
-      </c>
-      <c r="C3">
-        <v>1.74216027874564E-2</v>
-      </c>
-      <c r="D3">
-        <v>0.15331010452961599</v>
-      </c>
-      <c r="E3">
-        <v>0.23344947735191601</v>
-      </c>
-      <c r="F3">
-        <v>6.9686411149825697E-2</v>
-      </c>
-      <c r="G3">
-        <v>0.45993031358885</v>
-      </c>
-      <c r="H3">
-        <v>6.6202090592334395E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>494</v>
-      </c>
-      <c r="B4" t="s">
-        <v>478</v>
-      </c>
-      <c r="C4">
-        <v>1.5748031496062901E-3</v>
-      </c>
-      <c r="D4">
-        <v>0.97165354330708598</v>
-      </c>
-      <c r="E4">
-        <v>1.25984251968503E-2</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>1.5748031496062901E-3</v>
-      </c>
-      <c r="H4">
-        <v>1.25984251968503E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>495</v>
-      </c>
-      <c r="B5" t="s">
-        <v>481</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>8.7999999999999995E-2</v>
-      </c>
-      <c r="E5">
-        <v>1.6E-2</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0.42399999999999999</v>
-      </c>
-      <c r="H5">
-        <v>0.47199999999999998</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>496</v>
-      </c>
-      <c r="B6" t="s">
-        <v>478</v>
-      </c>
-      <c r="C6">
-        <v>3.20708613317043E-3</v>
-      </c>
-      <c r="D6">
-        <v>0.96525656689065298</v>
-      </c>
-      <c r="E6">
-        <v>7.4832009773976704E-3</v>
-      </c>
-      <c r="F6">
-        <v>2.0769700671960899E-2</v>
-      </c>
-      <c r="G6">
-        <v>3.0543677458766002E-3</v>
-      </c>
-      <c r="H6">
-        <v>2.29077580940745E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>497</v>
-      </c>
-      <c r="B7" t="s">
-        <v>481</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0.232876712328767</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0.56164383561643805</v>
-      </c>
-      <c r="H7">
-        <v>0.20547945205479401</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>498</v>
-      </c>
-      <c r="B8" t="s">
-        <v>478</v>
-      </c>
-      <c r="C8">
-        <v>0.237606590547767</v>
-      </c>
-      <c r="D8">
-        <v>4.3503396444572899E-2</v>
-      </c>
-      <c r="E8">
-        <v>0.64575805752276305</v>
-      </c>
-      <c r="F8">
-        <v>2.5003613238907301E-2</v>
-      </c>
-      <c r="G8">
-        <v>4.0612805318687599E-2</v>
-      </c>
-      <c r="H8">
-        <v>7.5155369273016302E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>499</v>
-      </c>
-      <c r="B9" t="s">
-        <v>481</v>
-      </c>
-      <c r="C9">
-        <v>0.165481443031404</v>
-      </c>
-      <c r="D9">
-        <v>2.34622372177524E-2</v>
-      </c>
-      <c r="E9">
-        <v>0.32561640280301002</v>
-      </c>
-      <c r="F9">
-        <v>8.7983389566571493E-2</v>
-      </c>
-      <c r="G9">
-        <v>6.3431092655073906E-2</v>
-      </c>
-      <c r="H9">
-        <v>0.33402543472618701</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>500</v>
-      </c>
-      <c r="B10" t="s">
-        <v>478</v>
-      </c>
-      <c r="C10">
-        <v>4.2270531400966102E-3</v>
-      </c>
-      <c r="D10">
-        <v>0.84118357487922701</v>
-      </c>
-      <c r="E10">
-        <v>1.1171497584541E-2</v>
-      </c>
-      <c r="F10">
-        <v>3.6231884057971002E-3</v>
-      </c>
-      <c r="G10">
-        <v>9.4907407407407399E-2</v>
-      </c>
-      <c r="H10">
-        <v>4.4887278582930699E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>501</v>
-      </c>
-      <c r="B11" t="s">
-        <v>481</v>
-      </c>
-      <c r="C11">
-        <v>3.54609929078014E-3</v>
-      </c>
-      <c r="D11">
-        <v>1.77304964539007E-2</v>
-      </c>
-      <c r="E11">
-        <v>0.29787234042553101</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0.53191489361702105</v>
-      </c>
-      <c r="H11">
-        <v>0.14893617021276501</v>
       </c>
     </row>
   </sheetData>
@@ -5376,2198 +6939,22 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3C70917-9931-D049-9BCD-DA2F45148023}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="7" max="7" width="16.5" customWidth="1"/>
-    <col min="8" max="8" width="14.1640625" customWidth="1"/>
-    <col min="9" max="9" width="15.5" customWidth="1"/>
-    <col min="10" max="10" width="17.5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>525</v>
-      </c>
-      <c r="B1" t="s">
-        <v>526</v>
-      </c>
-      <c r="C1" t="s">
-        <v>527</v>
-      </c>
-      <c r="D1" t="s">
-        <v>528</v>
-      </c>
-      <c r="E1" t="s">
-        <v>529</v>
-      </c>
-      <c r="F1" t="s">
-        <v>530</v>
-      </c>
-      <c r="G1" t="s">
-        <v>531</v>
-      </c>
-      <c r="H1" t="s">
-        <v>532</v>
-      </c>
-      <c r="I1" t="s">
-        <v>533</v>
-      </c>
-      <c r="J1" t="s">
-        <v>534</v>
-      </c>
-      <c r="K1" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>485</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>0.13642333904732401</v>
-      </c>
-      <c r="D2">
-        <v>0.22116298658184499</v>
-      </c>
-      <c r="E2">
-        <v>8.4739647534520401E-2</v>
-      </c>
-      <c r="F2">
-        <v>1.1171497584541E-2</v>
-      </c>
-      <c r="G2">
-        <v>0.23344947735191601</v>
-      </c>
-      <c r="H2">
-        <v>0.22539351135136901</v>
-      </c>
-      <c r="I2">
-        <v>5</v>
-      </c>
-      <c r="J2">
-        <v>0.625</v>
-      </c>
-      <c r="K2">
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>484</v>
-      </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>0.75456221185683803</v>
-      </c>
-      <c r="D3">
-        <v>5.65005676402539E-2</v>
-      </c>
-      <c r="E3">
-        <v>-0.69806164421658401</v>
-      </c>
-      <c r="F3">
-        <v>0.95121397776265004</v>
-      </c>
-      <c r="G3">
-        <v>2.34622372177524E-2</v>
-      </c>
-      <c r="H3">
-        <v>-0.823453078425326</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>6.25E-2</v>
-      </c>
-      <c r="K3">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>486</v>
-      </c>
-      <c r="B4">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1.1535756102089499E-2</v>
-      </c>
-      <c r="D4">
-        <v>3.1533960143279402E-2</v>
-      </c>
-      <c r="E4">
-        <v>1.99982040411898E-2</v>
-      </c>
-      <c r="F4">
-        <v>8.2822781937826103E-3</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>3</v>
-      </c>
-      <c r="J4">
-        <v>0.46520881845214102</v>
-      </c>
-      <c r="K4">
-        <v>0.55825058214256995</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>487</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>3.2227743754040999E-2</v>
-      </c>
-      <c r="D5">
-        <v>0.40818402709547602</v>
-      </c>
-      <c r="E5">
-        <v>0.37595628334143499</v>
-      </c>
-      <c r="F5">
-        <v>2.0989335148627102E-2</v>
-      </c>
-      <c r="G5">
-        <v>0.45993031358885</v>
-      </c>
-      <c r="H5">
-        <v>0.43700748620961299</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>6.25E-2</v>
-      </c>
-      <c r="K5">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>483</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <v>5.0298827038874998E-2</v>
-      </c>
-      <c r="D6">
-        <v>3.7289829021928102E-2</v>
-      </c>
-      <c r="E6">
-        <v>-1.30089980169469E-2</v>
-      </c>
-      <c r="F6">
-        <v>4.2270531400966102E-3</v>
-      </c>
-      <c r="G6">
-        <v>3.54609929078014E-3</v>
-      </c>
-      <c r="H6">
-        <v>-1.5748031496062901E-3</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6">
-        <v>0.4375</v>
-      </c>
-      <c r="K6">
-        <v>0.55825058214256995</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>488</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7">
-        <v>1.4952122200831299E-2</v>
-      </c>
-      <c r="D7">
-        <v>0.24532862951721601</v>
-      </c>
-      <c r="E7">
-        <v>0.23037650731638501</v>
-      </c>
-      <c r="F7">
-        <v>9.5302927161334192E-3</v>
-      </c>
-      <c r="G7">
-        <v>0.20547945205479401</v>
-      </c>
-      <c r="H7">
-        <v>0.205250374473853</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>6.25E-2</v>
-      </c>
-      <c r="K7">
-        <v>0.125</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B48EF9-98EE-9446-B8E9-8DACAA829D87}">
-  <dimension ref="A1:K100"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="32.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="B2" s="4">
-        <v>1</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="B3" s="4">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4">
-        <v>1</v>
-      </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5">
-        <v>1</v>
-      </c>
-      <c r="E4" s="5">
-        <v>1</v>
-      </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="B5" s="5">
-        <v>1</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5">
-        <v>1</v>
-      </c>
-      <c r="E5" s="5">
-        <v>1</v>
-      </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5">
-        <v>1</v>
-      </c>
-      <c r="I5" s="5">
-        <v>1</v>
-      </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5">
-        <v>1</v>
-      </c>
-      <c r="K6" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="B7" s="5">
-        <v>1</v>
-      </c>
-      <c r="C7" s="5">
-        <v>1</v>
-      </c>
-      <c r="D7" s="5">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5">
-        <v>1</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1</v>
-      </c>
-      <c r="G7" s="5">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5">
-        <v>1</v>
-      </c>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5">
-        <v>1</v>
-      </c>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4">
-        <v>1</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5">
-        <v>1</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5">
-        <v>1</v>
-      </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5">
-        <v>1</v>
-      </c>
-      <c r="I12" s="5">
-        <v>1</v>
-      </c>
-      <c r="J12" s="5">
-        <v>1</v>
-      </c>
-      <c r="K12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5">
-        <v>1</v>
-      </c>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="B15" s="5">
-        <v>1</v>
-      </c>
-      <c r="C15" s="5">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5">
-        <v>1</v>
-      </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5">
-        <v>1</v>
-      </c>
-      <c r="I16" s="5">
-        <v>1</v>
-      </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5">
-        <v>1</v>
-      </c>
-      <c r="D17" s="5">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5">
-        <v>1</v>
-      </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5">
-        <v>1</v>
-      </c>
-      <c r="H17" s="5">
-        <v>1</v>
-      </c>
-      <c r="I17" s="5">
-        <v>1</v>
-      </c>
-      <c r="J17" s="5">
-        <v>1</v>
-      </c>
-      <c r="K17" s="5"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5">
-        <v>1</v>
-      </c>
-      <c r="E18" s="5">
-        <v>1</v>
-      </c>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5">
-        <v>1</v>
-      </c>
-      <c r="H18" s="5">
-        <v>1</v>
-      </c>
-      <c r="I18" s="5">
-        <v>1</v>
-      </c>
-      <c r="J18" s="5">
-        <v>1</v>
-      </c>
-      <c r="K18" s="5"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="B19" s="5">
-        <v>1</v>
-      </c>
-      <c r="C19" s="5">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5">
-        <v>1</v>
-      </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5">
-        <v>1</v>
-      </c>
-      <c r="H19" s="5">
-        <v>1</v>
-      </c>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5">
-        <v>1</v>
-      </c>
-      <c r="K19" s="5"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5">
-        <v>1</v>
-      </c>
-      <c r="H20" s="5">
-        <v>1</v>
-      </c>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5">
-        <v>1</v>
-      </c>
-      <c r="K20" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>390</v>
-      </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5">
-        <v>1</v>
-      </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>391</v>
-      </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5">
-        <v>1</v>
-      </c>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="B23" s="5">
-        <v>1</v>
-      </c>
-      <c r="C23" s="5">
-        <v>1</v>
-      </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="B24" s="5">
-        <v>1</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5">
-        <v>1</v>
-      </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5">
-        <v>1</v>
-      </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5">
-        <v>1</v>
-      </c>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>396</v>
-      </c>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5">
-        <v>1</v>
-      </c>
-      <c r="E27" s="5">
-        <v>1</v>
-      </c>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5">
-        <v>1</v>
-      </c>
-      <c r="G28" s="5">
-        <v>1</v>
-      </c>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="B29" s="4">
-        <v>1</v>
-      </c>
-      <c r="C29" s="4">
-        <v>1</v>
-      </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
-        <v>399</v>
-      </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5">
-        <v>1</v>
-      </c>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5">
-        <v>1</v>
-      </c>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5">
-        <v>1</v>
-      </c>
-      <c r="K32" s="5"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="B34" s="5">
-        <v>1</v>
-      </c>
-      <c r="C34" s="5">
-        <v>1</v>
-      </c>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5">
-        <v>1</v>
-      </c>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="B36" s="5">
-        <v>1</v>
-      </c>
-      <c r="C36" s="5">
-        <v>1</v>
-      </c>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="B37" s="5">
-        <v>1</v>
-      </c>
-      <c r="C37" s="5">
-        <v>1</v>
-      </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5">
-        <v>1</v>
-      </c>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5">
-        <v>1</v>
-      </c>
-      <c r="I38" s="5">
-        <v>1</v>
-      </c>
-      <c r="J38" s="5">
-        <v>1</v>
-      </c>
-      <c r="K38" s="5"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5">
-        <v>1</v>
-      </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5">
-        <v>1</v>
-      </c>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5">
-        <v>1</v>
-      </c>
-      <c r="I39" s="5"/>
-      <c r="J39" s="5">
-        <v>1</v>
-      </c>
-      <c r="K39" s="5"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5">
-        <v>1</v>
-      </c>
-      <c r="D40" s="5">
-        <v>1</v>
-      </c>
-      <c r="E40" s="5">
-        <v>1</v>
-      </c>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5">
-        <v>1</v>
-      </c>
-      <c r="K40" s="5"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5">
-        <v>1</v>
-      </c>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5">
-        <v>1</v>
-      </c>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="5">
-        <v>1</v>
-      </c>
-      <c r="K41" s="5"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5">
-        <v>1</v>
-      </c>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5">
-        <v>1</v>
-      </c>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="5">
-        <v>1</v>
-      </c>
-      <c r="K42" s="5"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5">
-        <v>1</v>
-      </c>
-      <c r="D43" s="5">
-        <v>1</v>
-      </c>
-      <c r="E43" s="5">
-        <v>1</v>
-      </c>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-      <c r="I43" s="5"/>
-      <c r="J43" s="5"/>
-      <c r="K43" s="5"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5">
-        <v>1</v>
-      </c>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="I44" s="5"/>
-      <c r="J44" s="5"/>
-      <c r="K44" s="5"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5">
-        <v>1</v>
-      </c>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="B46" s="4">
-        <v>1</v>
-      </c>
-      <c r="C46" s="4">
-        <v>1</v>
-      </c>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-      <c r="J46" s="4"/>
-      <c r="K46" s="4"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5">
-        <v>1</v>
-      </c>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5">
-        <v>1</v>
-      </c>
-      <c r="I47" s="5"/>
-      <c r="J47" s="5">
-        <v>1</v>
-      </c>
-      <c r="K47" s="5"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5">
-        <v>1</v>
-      </c>
-      <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5">
-        <v>1</v>
-      </c>
-      <c r="G49" s="5">
-        <v>1</v>
-      </c>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
-        <v>421</v>
-      </c>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4">
-        <v>1</v>
-      </c>
-      <c r="E50" s="4">
-        <v>1</v>
-      </c>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
-        <v>423</v>
-      </c>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5">
-        <v>1</v>
-      </c>
-      <c r="I51" s="5">
-        <v>1</v>
-      </c>
-      <c r="J51" s="5"/>
-      <c r="K51" s="5"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="B52" s="4">
-        <v>1</v>
-      </c>
-      <c r="C52" s="4">
-        <v>1</v>
-      </c>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
-        <v>425</v>
-      </c>
-      <c r="B53" s="4">
-        <v>1</v>
-      </c>
-      <c r="C53" s="4">
-        <v>1</v>
-      </c>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
-      <c r="J53" s="4"/>
-      <c r="K53" s="4"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="B54" s="5"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5">
-        <v>1</v>
-      </c>
-      <c r="E54" s="5">
-        <v>1</v>
-      </c>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5"/>
-      <c r="I54" s="5"/>
-      <c r="J54" s="5"/>
-      <c r="K54" s="5"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A55" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-      <c r="J55" s="5">
-        <v>1</v>
-      </c>
-      <c r="K55" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="5"/>
-      <c r="I56" s="5"/>
-      <c r="J56" s="5">
-        <v>1</v>
-      </c>
-      <c r="K56" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="B57" s="4">
-        <v>1</v>
-      </c>
-      <c r="C57" s="4">
-        <v>1</v>
-      </c>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4">
-        <v>1</v>
-      </c>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A58" s="1" t="s">
-        <v>503</v>
-      </c>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
-      <c r="H58" s="5">
-        <v>1</v>
-      </c>
-      <c r="I58" s="5"/>
-      <c r="J58" s="5">
-        <v>1</v>
-      </c>
-      <c r="K58" s="5"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A59" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5">
-        <v>1</v>
-      </c>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-      <c r="I59" s="5">
-        <v>1</v>
-      </c>
-      <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="B60" s="4">
-        <v>1</v>
-      </c>
-      <c r="C60" s="4">
-        <v>1</v>
-      </c>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A61" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5">
-        <v>1</v>
-      </c>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5">
-        <v>1</v>
-      </c>
-      <c r="K61" s="5"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A62" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="B62" s="4">
-        <v>1</v>
-      </c>
-      <c r="C62" s="4">
-        <v>1</v>
-      </c>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-      <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A63" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5">
-        <v>1</v>
-      </c>
-      <c r="E63" s="5">
-        <v>1</v>
-      </c>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
-        <v>437</v>
-      </c>
-      <c r="B64" s="4">
-        <v>1</v>
-      </c>
-      <c r="C64" s="4">
-        <v>1</v>
-      </c>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
-        <v>438</v>
-      </c>
-      <c r="B65" s="4"/>
-      <c r="C65" s="4">
-        <v>1</v>
-      </c>
-      <c r="D65" s="4"/>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-      <c r="I65" s="4"/>
-      <c r="J65" s="4"/>
-      <c r="K65" s="4"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A66" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5">
-        <v>1</v>
-      </c>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
-      <c r="G66" s="5"/>
-      <c r="H66" s="5"/>
-      <c r="I66" s="5"/>
-      <c r="J66" s="5"/>
-      <c r="K66" s="5"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A67" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5">
-        <v>1</v>
-      </c>
-      <c r="K67" s="5"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A68" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-      <c r="G68" s="5"/>
-      <c r="H68" s="5">
-        <v>1</v>
-      </c>
-      <c r="I68" s="5"/>
-      <c r="J68" s="5"/>
-      <c r="K68" s="5"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A69" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
-      <c r="H69" s="5"/>
-      <c r="I69" s="5"/>
-      <c r="J69" s="5">
-        <v>1</v>
-      </c>
-      <c r="K69" s="5"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A70" s="1" t="s">
-        <v>444</v>
-      </c>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5">
-        <v>1</v>
-      </c>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
-      <c r="H70" s="5"/>
-      <c r="I70" s="5"/>
-      <c r="J70" s="5"/>
-      <c r="K70" s="5"/>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A71" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5">
-        <v>1</v>
-      </c>
-      <c r="D71" s="5"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
-      <c r="H71" s="5"/>
-      <c r="I71" s="5"/>
-      <c r="J71" s="5"/>
-      <c r="K71" s="5"/>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A72" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5">
-        <v>1</v>
-      </c>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
-      <c r="H72" s="5"/>
-      <c r="I72" s="5"/>
-      <c r="J72" s="5"/>
-      <c r="K72" s="5"/>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A73" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="B73" s="5"/>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
-      <c r="F73" s="5"/>
-      <c r="G73" s="5"/>
-      <c r="H73" s="5"/>
-      <c r="I73" s="5"/>
-      <c r="J73" s="5">
-        <v>1</v>
-      </c>
-      <c r="K73" s="5"/>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A74" s="1" t="s">
-        <v>509</v>
-      </c>
-      <c r="B74" s="5"/>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5">
-        <v>1</v>
-      </c>
-      <c r="G74" s="5"/>
-      <c r="H74" s="5"/>
-      <c r="I74" s="5"/>
-      <c r="J74" s="5"/>
-      <c r="K74" s="5"/>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A75" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="B75" s="5"/>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
-      <c r="G75" s="5"/>
-      <c r="H75" s="5">
-        <v>1</v>
-      </c>
-      <c r="I75" s="5"/>
-      <c r="J75" s="5"/>
-      <c r="K75" s="5"/>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A76" s="1" t="s">
-        <v>450</v>
-      </c>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
-      <c r="H76" s="5">
-        <v>1</v>
-      </c>
-      <c r="I76" s="5"/>
-      <c r="J76" s="5"/>
-      <c r="K76" s="5"/>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A77" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="5"/>
-      <c r="F77" s="5"/>
-      <c r="G77" s="5">
-        <v>1</v>
-      </c>
-      <c r="H77" s="5"/>
-      <c r="I77" s="5"/>
-      <c r="J77" s="5"/>
-      <c r="K77" s="5"/>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A78" s="1" t="s">
-        <v>510</v>
-      </c>
-      <c r="B78" s="5"/>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
-      <c r="G78" s="5">
-        <v>1</v>
-      </c>
-      <c r="H78" s="5"/>
-      <c r="I78" s="5"/>
-      <c r="J78" s="5"/>
-      <c r="K78" s="5"/>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A79" s="1" t="s">
-        <v>453</v>
-      </c>
-      <c r="B79" s="5"/>
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="5"/>
-      <c r="F79" s="5"/>
-      <c r="G79" s="5"/>
-      <c r="H79" s="5">
-        <v>1</v>
-      </c>
-      <c r="I79" s="5"/>
-      <c r="J79" s="5"/>
-      <c r="K79" s="5"/>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A80" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="B80" s="5"/>
-      <c r="C80" s="5"/>
-      <c r="D80" s="5"/>
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-      <c r="G80" s="5"/>
-      <c r="H80" s="5"/>
-      <c r="I80" s="5">
-        <v>1</v>
-      </c>
-      <c r="J80" s="5"/>
-      <c r="K80" s="5"/>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A81" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="B81" s="5"/>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-      <c r="G81" s="5"/>
-      <c r="H81" s="5"/>
-      <c r="I81" s="5"/>
-      <c r="J81" s="5">
-        <v>1</v>
-      </c>
-      <c r="K81" s="5"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A82" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="B82" s="5"/>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
-      <c r="G82" s="5"/>
-      <c r="H82" s="5"/>
-      <c r="I82" s="5"/>
-      <c r="J82" s="5"/>
-      <c r="K82" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A83" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="B83" s="5"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-      <c r="G83" s="5"/>
-      <c r="H83" s="5">
-        <v>1</v>
-      </c>
-      <c r="I83" s="5">
-        <v>1</v>
-      </c>
-      <c r="J83" s="5"/>
-      <c r="K83" s="5"/>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A84" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="B84" s="5">
-        <v>1</v>
-      </c>
-      <c r="C84" s="5">
-        <v>1</v>
-      </c>
-      <c r="D84" s="5"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-      <c r="G84" s="5"/>
-      <c r="H84" s="5"/>
-      <c r="I84" s="5"/>
-      <c r="J84" s="5"/>
-      <c r="K84" s="5"/>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A85" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="B85" s="5"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5">
-        <v>1</v>
-      </c>
-      <c r="E85" s="5">
-        <v>1</v>
-      </c>
-      <c r="F85" s="5"/>
-      <c r="G85" s="5"/>
-      <c r="H85" s="5"/>
-      <c r="I85" s="5"/>
-      <c r="J85" s="5"/>
-      <c r="K85" s="5"/>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A86" s="1" t="s">
-        <v>511</v>
-      </c>
-      <c r="B86" s="5"/>
-      <c r="C86" s="5"/>
-      <c r="D86" s="5">
-        <v>1</v>
-      </c>
-      <c r="E86" s="5">
-        <v>1</v>
-      </c>
-      <c r="F86" s="5"/>
-      <c r="G86" s="5"/>
-      <c r="H86" s="5"/>
-      <c r="I86" s="5"/>
-      <c r="J86" s="5"/>
-      <c r="K86" s="5"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A87" s="3" t="s">
-        <v>462</v>
-      </c>
-      <c r="B87" s="4">
-        <v>1</v>
-      </c>
-      <c r="C87" s="4">
-        <v>1</v>
-      </c>
-      <c r="D87" s="4"/>
-      <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
-      <c r="H87" s="4"/>
-      <c r="I87" s="4"/>
-      <c r="J87" s="4"/>
-      <c r="K87" s="4"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A88" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="B88" s="5"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="5">
-        <v>1</v>
-      </c>
-      <c r="E88" s="5"/>
-      <c r="F88" s="5"/>
-      <c r="G88" s="5"/>
-      <c r="H88" s="5"/>
-      <c r="I88" s="5"/>
-      <c r="J88" s="5"/>
-      <c r="K88" s="5"/>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A89" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="B89" s="5"/>
-      <c r="C89" s="5"/>
-      <c r="D89" s="5"/>
-      <c r="E89" s="5">
-        <v>1</v>
-      </c>
-      <c r="F89" s="5"/>
-      <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
-      <c r="I89" s="5"/>
-      <c r="J89" s="5"/>
-      <c r="K89" s="5"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A90" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5">
-        <v>1</v>
-      </c>
-      <c r="D90" s="5"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
-      <c r="G90" s="5"/>
-      <c r="H90" s="5"/>
-      <c r="I90" s="5"/>
-      <c r="J90" s="5"/>
-      <c r="K90" s="5"/>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A91" s="1" t="s">
-        <v>514</v>
-      </c>
-      <c r="B91" s="5"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="5"/>
-      <c r="E91" s="5"/>
-      <c r="F91" s="5"/>
-      <c r="G91" s="5"/>
-      <c r="H91" s="5"/>
-      <c r="I91" s="5"/>
-      <c r="J91" s="5">
-        <v>1</v>
-      </c>
-      <c r="K91" s="5"/>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A92" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="B92" s="5"/>
-      <c r="C92" s="5"/>
-      <c r="D92" s="5"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="5"/>
-      <c r="G92" s="5"/>
-      <c r="H92" s="5">
-        <v>1</v>
-      </c>
-      <c r="I92" s="5"/>
-      <c r="J92" s="5"/>
-      <c r="K92" s="5"/>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A93" s="1" t="s">
-        <v>515</v>
-      </c>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="5"/>
-      <c r="E93" s="5"/>
-      <c r="F93" s="5"/>
-      <c r="G93" s="5"/>
-      <c r="H93" s="5">
-        <v>1</v>
-      </c>
-      <c r="I93" s="5"/>
-      <c r="J93" s="5"/>
-      <c r="K93" s="5"/>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A94" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="B94" s="5"/>
-      <c r="C94" s="5"/>
-      <c r="D94" s="5"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
-      <c r="G94" s="5"/>
-      <c r="H94" s="5"/>
-      <c r="I94" s="5"/>
-      <c r="J94" s="5">
-        <v>1</v>
-      </c>
-      <c r="K94" s="5"/>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A95" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="B95" s="5">
-        <v>1</v>
-      </c>
-      <c r="C95" s="5">
-        <v>1</v>
-      </c>
-      <c r="D95" s="5"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="5"/>
-      <c r="G95" s="5"/>
-      <c r="H95" s="5"/>
-      <c r="I95" s="5"/>
-      <c r="J95" s="5"/>
-      <c r="K95" s="5"/>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A96" s="1" t="s">
-        <v>517</v>
-      </c>
-      <c r="B96" s="5"/>
-      <c r="C96" s="5"/>
-      <c r="D96" s="5"/>
-      <c r="E96" s="5"/>
-      <c r="F96" s="5"/>
-      <c r="G96" s="5"/>
-      <c r="H96" s="5">
-        <v>1</v>
-      </c>
-      <c r="I96" s="5"/>
-      <c r="J96" s="5"/>
-      <c r="K96" s="5"/>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A97" s="1" t="s">
-        <v>518</v>
-      </c>
-      <c r="B97" s="5"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="5">
-        <v>1</v>
-      </c>
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5"/>
-      <c r="H97" s="5"/>
-      <c r="I97" s="5"/>
-      <c r="J97" s="5"/>
-      <c r="K97" s="5"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A98" s="1" t="s">
-        <v>519</v>
-      </c>
-      <c r="B98" s="5"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="5"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
-      <c r="G98" s="5"/>
-      <c r="H98" s="5"/>
-      <c r="I98" s="5"/>
-      <c r="J98" s="5">
-        <v>1</v>
-      </c>
-      <c r="K98" s="5"/>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A99" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="B99" s="5"/>
-      <c r="C99" s="5"/>
-      <c r="D99" s="5"/>
-      <c r="E99" s="5"/>
-      <c r="F99" s="5"/>
-      <c r="G99" s="5"/>
-      <c r="H99" s="5">
-        <v>1</v>
-      </c>
-      <c r="I99" s="5"/>
-      <c r="J99" s="5"/>
-      <c r="K99" s="5"/>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A100" s="1" t="s">
-        <v>520</v>
-      </c>
-      <c r="B100" s="5"/>
-      <c r="C100" s="5"/>
-      <c r="D100" s="5"/>
-      <c r="E100" s="5"/>
-      <c r="F100" s="5"/>
-      <c r="G100" s="5">
-        <v>1</v>
-      </c>
-      <c r="H100" s="5"/>
-      <c r="I100" s="5"/>
-      <c r="J100" s="5"/>
-      <c r="K100" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{099D8DB7-1C01-8040-BBF1-2F2FE6508470}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="B1" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="C1" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="D1" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update analysis scripts, figures, and source data
</commit_message>
<xml_diff>
--- a/manu_sourcedata/suppl_tables.xlsx
+++ b/manu_sourcedata/suppl_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manu_sourcedata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089507A9-F083-734B-BEC0-A43340A448B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE61B1A-357B-C246-BD74-A2A416C5E8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7900" yWindow="-28300" windowWidth="33680" windowHeight="12580" activeTab="2" xr2:uid="{07063887-18E2-9747-8ACB-521C19DAFDA2}"/>
+    <workbookView xWindow="37580" yWindow="-440" windowWidth="34560" windowHeight="21100" xr2:uid="{07063887-18E2-9747-8ACB-521C19DAFDA2}"/>
   </bookViews>
   <sheets>
     <sheet name="1 TCR probes and samples" sheetId="4" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="3 ind T cell subtype prop" sheetId="2" r:id="rId3"/>
     <sheet name="4 filtered gene lists" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="522">
   <si>
     <t>CDH19</t>
   </si>
@@ -1957,12 +1957,21 @@
   <si>
     <t>Proliferating T</t>
   </si>
+  <si>
+    <t>Criteria 3</t>
+  </si>
+  <si>
+    <t>Criteria 2</t>
+  </si>
+  <si>
+    <t>Criteria 1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1987,6 +1996,13 @@
       <color theme="1"/>
       <name val="Aptos Narrow (Body)"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2008,7 +2024,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2025,6 +2041,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2359,13 +2376,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B48EF9-98EE-9446-B8E9-8DACAA829D87}">
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:N100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>494</v>
       </c>
@@ -2399,8 +2416,17 @@
       <c r="K1" s="2" t="s">
         <v>493</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>389</v>
       </c>
@@ -2418,8 +2444,17 @@
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>400</v>
       </c>
@@ -2437,8 +2472,17 @@
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>411</v>
       </c>
@@ -2456,8 +2500,17 @@
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>422</v>
       </c>
@@ -2483,8 +2536,17 @@
       </c>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>432</v>
       </c>
@@ -2502,8 +2564,17 @@
       <c r="K6" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>443</v>
       </c>
@@ -2533,8 +2604,17 @@
         <v>1</v>
       </c>
       <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>454</v>
       </c>
@@ -2550,8 +2630,17 @@
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="b">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>465</v>
       </c>
@@ -2567,8 +2656,17 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>476</v>
       </c>
@@ -2584,8 +2682,17 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>379</v>
       </c>
@@ -2601,8 +2708,17 @@
       </c>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>380</v>
       </c>
@@ -2622,8 +2738,17 @@
         <v>1</v>
       </c>
       <c r="K12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N12" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>381</v>
       </c>
@@ -2639,8 +2764,17 @@
       <c r="K13" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" t="b">
+        <v>0</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>382</v>
       </c>
@@ -2656,8 +2790,17 @@
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" t="b">
+        <v>0</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>383</v>
       </c>
@@ -2675,8 +2818,17 @@
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>384</v>
       </c>
@@ -2698,8 +2850,17 @@
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="b">
+        <v>1</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>385</v>
       </c>
@@ -2727,8 +2888,17 @@
         <v>1</v>
       </c>
       <c r="K17" s="5"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
+      </c>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>386</v>
       </c>
@@ -2754,8 +2924,17 @@
         <v>1</v>
       </c>
       <c r="K18" s="5"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" t="b">
+        <v>1</v>
+      </c>
+      <c r="N18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>387</v>
       </c>
@@ -2781,8 +2960,17 @@
         <v>1</v>
       </c>
       <c r="K19" s="5"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="b">
+        <v>1</v>
+      </c>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>388</v>
       </c>
@@ -2806,8 +2994,17 @@
       <c r="K20" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M20" t="b">
+        <v>1</v>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>390</v>
       </c>
@@ -2823,8 +3020,17 @@
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" t="b">
+        <v>0</v>
+      </c>
+      <c r="N21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>391</v>
       </c>
@@ -2840,8 +3046,17 @@
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="b">
+        <v>0</v>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>392</v>
       </c>
@@ -2859,8 +3074,17 @@
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="b">
+        <v>0</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>393</v>
       </c>
@@ -2876,8 +3100,17 @@
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" t="b">
+        <v>0</v>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>394</v>
       </c>
@@ -2893,8 +3126,17 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
       <c r="K25" s="5"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
+      <c r="M25" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>395</v>
       </c>
@@ -2912,8 +3154,17 @@
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
       <c r="K26" s="5"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" t="b">
+        <v>1</v>
+      </c>
+      <c r="M26" t="b">
+        <v>1</v>
+      </c>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>396</v>
       </c>
@@ -2931,8 +3182,17 @@
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
+      <c r="M27" t="b">
+        <v>0</v>
+      </c>
+      <c r="N27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>397</v>
       </c>
@@ -2950,8 +3210,17 @@
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28" t="b">
+        <v>0</v>
+      </c>
+      <c r="M28" t="b">
+        <v>0</v>
+      </c>
+      <c r="N28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>398</v>
       </c>
@@ -2969,8 +3238,17 @@
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
+      <c r="M29" t="b">
+        <v>0</v>
+      </c>
+      <c r="N29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>399</v>
       </c>
@@ -2986,8 +3264,17 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
+      <c r="M30" t="b">
+        <v>0</v>
+      </c>
+      <c r="N30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>401</v>
       </c>
@@ -3003,8 +3290,17 @@
       </c>
       <c r="J31" s="5"/>
       <c r="K31" s="5"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L31" t="b">
+        <v>0</v>
+      </c>
+      <c r="M31" t="b">
+        <v>0</v>
+      </c>
+      <c r="N31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>402</v>
       </c>
@@ -3020,8 +3316,17 @@
         <v>1</v>
       </c>
       <c r="K32" s="5"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L32" t="b">
+        <v>1</v>
+      </c>
+      <c r="M32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>403</v>
       </c>
@@ -3037,8 +3342,17 @@
       <c r="K33" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>404</v>
       </c>
@@ -3056,8 +3370,17 @@
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
       <c r="K34" s="5"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" t="b">
+        <v>1</v>
+      </c>
+      <c r="M34" t="b">
+        <v>0</v>
+      </c>
+      <c r="N34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>405</v>
       </c>
@@ -3073,8 +3396,17 @@
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L35" t="b">
+        <v>1</v>
+      </c>
+      <c r="M35" t="b">
+        <v>0</v>
+      </c>
+      <c r="N35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>406</v>
       </c>
@@ -3092,8 +3424,17 @@
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
       <c r="K36" s="5"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L36" t="b">
+        <v>1</v>
+      </c>
+      <c r="M36" t="b">
+        <v>0</v>
+      </c>
+      <c r="N36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>407</v>
       </c>
@@ -3111,8 +3452,17 @@
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="5"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L37" t="b">
+        <v>1</v>
+      </c>
+      <c r="M37" t="b">
+        <v>0</v>
+      </c>
+      <c r="N37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>408</v>
       </c>
@@ -3134,8 +3484,17 @@
         <v>1</v>
       </c>
       <c r="K38" s="5"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L38" t="b">
+        <v>1</v>
+      </c>
+      <c r="M38" t="b">
+        <v>1</v>
+      </c>
+      <c r="N38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>409</v>
       </c>
@@ -3157,8 +3516,17 @@
         <v>1</v>
       </c>
       <c r="K39" s="5"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L39" t="b">
+        <v>1</v>
+      </c>
+      <c r="M39" t="b">
+        <v>1</v>
+      </c>
+      <c r="N39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>410</v>
       </c>
@@ -3180,8 +3548,17 @@
         <v>1</v>
       </c>
       <c r="K40" s="5"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L40" t="b">
+        <v>0</v>
+      </c>
+      <c r="M40" t="b">
+        <v>1</v>
+      </c>
+      <c r="N40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>412</v>
       </c>
@@ -3201,8 +3578,17 @@
         <v>1</v>
       </c>
       <c r="K41" s="5"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L41" t="b">
+        <v>0</v>
+      </c>
+      <c r="M41" t="b">
+        <v>1</v>
+      </c>
+      <c r="N41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>413</v>
       </c>
@@ -3222,8 +3608,17 @@
         <v>1</v>
       </c>
       <c r="K42" s="5"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L42" t="b">
+        <v>0</v>
+      </c>
+      <c r="M42" t="b">
+        <v>1</v>
+      </c>
+      <c r="N42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>414</v>
       </c>
@@ -3243,8 +3638,17 @@
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
+      <c r="M43" t="b">
+        <v>1</v>
+      </c>
+      <c r="N43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>415</v>
       </c>
@@ -3260,8 +3664,17 @@
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L44" t="b">
+        <v>1</v>
+      </c>
+      <c r="M44" t="b">
+        <v>0</v>
+      </c>
+      <c r="N44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>416</v>
       </c>
@@ -3277,8 +3690,17 @@
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L45" t="b">
+        <v>1</v>
+      </c>
+      <c r="M45" t="b">
+        <v>0</v>
+      </c>
+      <c r="N45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>417</v>
       </c>
@@ -3296,8 +3718,17 @@
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
       <c r="K46" s="4"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L46" t="b">
+        <v>1</v>
+      </c>
+      <c r="M46" t="b">
+        <v>0</v>
+      </c>
+      <c r="N46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>418</v>
       </c>
@@ -3317,8 +3748,17 @@
         <v>1</v>
       </c>
       <c r="K47" s="5"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L47" t="b">
+        <v>1</v>
+      </c>
+      <c r="M47" t="b">
+        <v>1</v>
+      </c>
+      <c r="N47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>419</v>
       </c>
@@ -3336,8 +3776,17 @@
       <c r="K48" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L48" t="b">
+        <v>0</v>
+      </c>
+      <c r="M48" t="b">
+        <v>1</v>
+      </c>
+      <c r="N48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>420</v>
       </c>
@@ -3355,8 +3804,17 @@
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L49" t="b">
+        <v>0</v>
+      </c>
+      <c r="M49" t="b">
+        <v>0</v>
+      </c>
+      <c r="N49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>421</v>
       </c>
@@ -3374,8 +3832,17 @@
       <c r="I50" s="4"/>
       <c r="J50" s="4"/>
       <c r="K50" s="4"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L50" t="b">
+        <v>0</v>
+      </c>
+      <c r="M50" t="b">
+        <v>0</v>
+      </c>
+      <c r="N50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>423</v>
       </c>
@@ -3393,8 +3860,17 @@
       </c>
       <c r="J51" s="5"/>
       <c r="K51" s="5"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L51" t="b">
+        <v>0</v>
+      </c>
+      <c r="M51" t="b">
+        <v>0</v>
+      </c>
+      <c r="N51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>424</v>
       </c>
@@ -3412,8 +3888,17 @@
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
       <c r="K52" s="4"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L52" t="b">
+        <v>0</v>
+      </c>
+      <c r="M52" t="b">
+        <v>0</v>
+      </c>
+      <c r="N52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>425</v>
       </c>
@@ -3431,8 +3916,17 @@
       <c r="I53" s="4"/>
       <c r="J53" s="4"/>
       <c r="K53" s="4"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L53" t="b">
+        <v>1</v>
+      </c>
+      <c r="M53" t="b">
+        <v>0</v>
+      </c>
+      <c r="N53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>426</v>
       </c>
@@ -3450,8 +3944,17 @@
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
       <c r="K54" s="5"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L54" t="b">
+        <v>0</v>
+      </c>
+      <c r="M54" t="b">
+        <v>0</v>
+      </c>
+      <c r="N54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>427</v>
       </c>
@@ -3469,8 +3972,17 @@
       <c r="K55" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L55" t="b">
+        <v>0</v>
+      </c>
+      <c r="M55" t="b">
+        <v>0</v>
+      </c>
+      <c r="N55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>428</v>
       </c>
@@ -3488,8 +4000,17 @@
       <c r="K56" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L56" t="b">
+        <v>1</v>
+      </c>
+      <c r="M56" t="b">
+        <v>0</v>
+      </c>
+      <c r="N56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>429</v>
       </c>
@@ -3509,8 +4030,17 @@
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
       <c r="K57" s="4"/>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L57" t="b">
+        <v>1</v>
+      </c>
+      <c r="M57" t="b">
+        <v>1</v>
+      </c>
+      <c r="N57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>495</v>
       </c>
@@ -3528,8 +4058,17 @@
         <v>1</v>
       </c>
       <c r="K58" s="5"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L58" t="b">
+        <v>0</v>
+      </c>
+      <c r="M58" t="b">
+        <v>1</v>
+      </c>
+      <c r="N58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>431</v>
       </c>
@@ -3547,8 +4086,17 @@
       </c>
       <c r="J59" s="5"/>
       <c r="K59" s="5"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L59" t="b">
+        <v>0</v>
+      </c>
+      <c r="M59" t="b">
+        <v>1</v>
+      </c>
+      <c r="N59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>433</v>
       </c>
@@ -3566,8 +4114,17 @@
       <c r="I60" s="4"/>
       <c r="J60" s="4"/>
       <c r="K60" s="4"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L60" t="b">
+        <v>1</v>
+      </c>
+      <c r="M60" t="b">
+        <v>0</v>
+      </c>
+      <c r="N60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>434</v>
       </c>
@@ -3585,8 +4142,17 @@
         <v>1</v>
       </c>
       <c r="K61" s="5"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L61" t="b">
+        <v>0</v>
+      </c>
+      <c r="M61" t="b">
+        <v>1</v>
+      </c>
+      <c r="N61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>435</v>
       </c>
@@ -3604,8 +4170,17 @@
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
       <c r="K62" s="4"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L62" t="b">
+        <v>0</v>
+      </c>
+      <c r="M62" t="b">
+        <v>0</v>
+      </c>
+      <c r="N62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>436</v>
       </c>
@@ -3623,8 +4198,17 @@
       <c r="I63" s="5"/>
       <c r="J63" s="5"/>
       <c r="K63" s="5"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L63" t="b">
+        <v>1</v>
+      </c>
+      <c r="M63" t="b">
+        <v>0</v>
+      </c>
+      <c r="N63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>437</v>
       </c>
@@ -3642,8 +4226,17 @@
       <c r="I64" s="4"/>
       <c r="J64" s="4"/>
       <c r="K64" s="4"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L64" t="b">
+        <v>1</v>
+      </c>
+      <c r="M64" t="b">
+        <v>0</v>
+      </c>
+      <c r="N64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>438</v>
       </c>
@@ -3659,8 +4252,17 @@
       <c r="I65" s="4"/>
       <c r="J65" s="4"/>
       <c r="K65" s="4"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L65" t="b">
+        <v>1</v>
+      </c>
+      <c r="M65" t="b">
+        <v>0</v>
+      </c>
+      <c r="N65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>439</v>
       </c>
@@ -3676,8 +4278,17 @@
       <c r="I66" s="5"/>
       <c r="J66" s="5"/>
       <c r="K66" s="5"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L66" t="b">
+        <v>1</v>
+      </c>
+      <c r="M66" t="b">
+        <v>0</v>
+      </c>
+      <c r="N66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>440</v>
       </c>
@@ -3693,8 +4304,17 @@
         <v>1</v>
       </c>
       <c r="K67" s="5"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L67" t="b">
+        <v>0</v>
+      </c>
+      <c r="M67" t="b">
+        <v>0</v>
+      </c>
+      <c r="N67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>496</v>
       </c>
@@ -3710,8 +4330,17 @@
       <c r="I68" s="5"/>
       <c r="J68" s="5"/>
       <c r="K68" s="5"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L68" t="b">
+        <v>0</v>
+      </c>
+      <c r="M68" t="b">
+        <v>0</v>
+      </c>
+      <c r="N68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>497</v>
       </c>
@@ -3727,8 +4356,17 @@
         <v>1</v>
       </c>
       <c r="K69" s="5"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L69" t="b">
+        <v>0</v>
+      </c>
+      <c r="M69" t="b">
+        <v>0</v>
+      </c>
+      <c r="N69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>444</v>
       </c>
@@ -3744,8 +4382,17 @@
       <c r="I70" s="5"/>
       <c r="J70" s="5"/>
       <c r="K70" s="5"/>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L70" t="b">
+        <v>0</v>
+      </c>
+      <c r="M70" t="b">
+        <v>0</v>
+      </c>
+      <c r="N70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>498</v>
       </c>
@@ -3761,8 +4408,17 @@
       <c r="I71" s="5"/>
       <c r="J71" s="5"/>
       <c r="K71" s="5"/>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L71" t="b">
+        <v>0</v>
+      </c>
+      <c r="M71" t="b">
+        <v>0</v>
+      </c>
+      <c r="N71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>499</v>
       </c>
@@ -3778,8 +4434,17 @@
       <c r="I72" s="5"/>
       <c r="J72" s="5"/>
       <c r="K72" s="5"/>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L72" t="b">
+        <v>0</v>
+      </c>
+      <c r="M72" t="b">
+        <v>0</v>
+      </c>
+      <c r="N72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>500</v>
       </c>
@@ -3795,8 +4460,17 @@
         <v>1</v>
       </c>
       <c r="K73" s="5"/>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L73" t="b">
+        <v>0</v>
+      </c>
+      <c r="M73" t="b">
+        <v>0</v>
+      </c>
+      <c r="N73" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>501</v>
       </c>
@@ -3812,8 +4486,17 @@
       <c r="I74" s="5"/>
       <c r="J74" s="5"/>
       <c r="K74" s="5"/>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L74" t="b">
+        <v>0</v>
+      </c>
+      <c r="M74" t="b">
+        <v>0</v>
+      </c>
+      <c r="N74" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>449</v>
       </c>
@@ -3829,8 +4512,17 @@
       <c r="I75" s="5"/>
       <c r="J75" s="5"/>
       <c r="K75" s="5"/>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L75" t="b">
+        <v>0</v>
+      </c>
+      <c r="M75" t="b">
+        <v>0</v>
+      </c>
+      <c r="N75" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>450</v>
       </c>
@@ -3846,8 +4538,17 @@
       <c r="I76" s="5"/>
       <c r="J76" s="5"/>
       <c r="K76" s="5"/>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L76" t="b">
+        <v>0</v>
+      </c>
+      <c r="M76" t="b">
+        <v>0</v>
+      </c>
+      <c r="N76" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>451</v>
       </c>
@@ -3863,8 +4564,17 @@
       <c r="I77" s="5"/>
       <c r="J77" s="5"/>
       <c r="K77" s="5"/>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L77" t="b">
+        <v>0</v>
+      </c>
+      <c r="M77" t="b">
+        <v>0</v>
+      </c>
+      <c r="N77" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>502</v>
       </c>
@@ -3880,8 +4590,17 @@
       <c r="I78" s="5"/>
       <c r="J78" s="5"/>
       <c r="K78" s="5"/>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L78" t="b">
+        <v>0</v>
+      </c>
+      <c r="M78" t="b">
+        <v>0</v>
+      </c>
+      <c r="N78" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>453</v>
       </c>
@@ -3897,8 +4616,17 @@
       <c r="I79" s="5"/>
       <c r="J79" s="5"/>
       <c r="K79" s="5"/>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L79" t="b">
+        <v>0</v>
+      </c>
+      <c r="M79" t="b">
+        <v>0</v>
+      </c>
+      <c r="N79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>455</v>
       </c>
@@ -3914,8 +4642,17 @@
       </c>
       <c r="J80" s="5"/>
       <c r="K80" s="5"/>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L80" t="b">
+        <v>0</v>
+      </c>
+      <c r="M80" t="b">
+        <v>0</v>
+      </c>
+      <c r="N80" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>456</v>
       </c>
@@ -3931,8 +4668,17 @@
         <v>1</v>
       </c>
       <c r="K81" s="5"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L81" t="b">
+        <v>0</v>
+      </c>
+      <c r="M81" t="b">
+        <v>0</v>
+      </c>
+      <c r="N81" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>457</v>
       </c>
@@ -3948,8 +4694,17 @@
       <c r="K82" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L82" t="b">
+        <v>0</v>
+      </c>
+      <c r="M82" t="b">
+        <v>0</v>
+      </c>
+      <c r="N82" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>458</v>
       </c>
@@ -3967,8 +4722,17 @@
       </c>
       <c r="J83" s="5"/>
       <c r="K83" s="5"/>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L83" t="b">
+        <v>0</v>
+      </c>
+      <c r="M83" t="b">
+        <v>0</v>
+      </c>
+      <c r="N83" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>459</v>
       </c>
@@ -3986,8 +4750,17 @@
       <c r="I84" s="5"/>
       <c r="J84" s="5"/>
       <c r="K84" s="5"/>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L84" t="b">
+        <v>0</v>
+      </c>
+      <c r="M84" t="b">
+        <v>0</v>
+      </c>
+      <c r="N84" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>460</v>
       </c>
@@ -4005,8 +4778,17 @@
       <c r="I85" s="5"/>
       <c r="J85" s="5"/>
       <c r="K85" s="5"/>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L85" t="b">
+        <v>0</v>
+      </c>
+      <c r="M85" t="b">
+        <v>0</v>
+      </c>
+      <c r="N85" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>503</v>
       </c>
@@ -4024,8 +4806,17 @@
       <c r="I86" s="5"/>
       <c r="J86" s="5"/>
       <c r="K86" s="5"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L86" t="b">
+        <v>0</v>
+      </c>
+      <c r="M86" t="b">
+        <v>0</v>
+      </c>
+      <c r="N86" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
         <v>462</v>
       </c>
@@ -4043,8 +4834,17 @@
       <c r="I87" s="4"/>
       <c r="J87" s="4"/>
       <c r="K87" s="4"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L87" t="b">
+        <v>0</v>
+      </c>
+      <c r="M87" t="b">
+        <v>0</v>
+      </c>
+      <c r="N87" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>504</v>
       </c>
@@ -4060,8 +4860,17 @@
       <c r="I88" s="5"/>
       <c r="J88" s="5"/>
       <c r="K88" s="5"/>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L88" t="b">
+        <v>0</v>
+      </c>
+      <c r="M88" t="b">
+        <v>0</v>
+      </c>
+      <c r="N88" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>464</v>
       </c>
@@ -4077,8 +4886,17 @@
       <c r="I89" s="5"/>
       <c r="J89" s="5"/>
       <c r="K89" s="5"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L89" t="b">
+        <v>0</v>
+      </c>
+      <c r="M89" t="b">
+        <v>0</v>
+      </c>
+      <c r="N89" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>505</v>
       </c>
@@ -4094,8 +4912,17 @@
       <c r="I90" s="5"/>
       <c r="J90" s="5"/>
       <c r="K90" s="5"/>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L90" t="b">
+        <v>1</v>
+      </c>
+      <c r="M90" t="b">
+        <v>0</v>
+      </c>
+      <c r="N90" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>506</v>
       </c>
@@ -4111,8 +4938,17 @@
         <v>1</v>
       </c>
       <c r="K91" s="5"/>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L91" t="b">
+        <v>0</v>
+      </c>
+      <c r="M91" t="b">
+        <v>0</v>
+      </c>
+      <c r="N91" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>468</v>
       </c>
@@ -4128,8 +4964,17 @@
       <c r="I92" s="5"/>
       <c r="J92" s="5"/>
       <c r="K92" s="5"/>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L92" t="b">
+        <v>0</v>
+      </c>
+      <c r="M92" t="b">
+        <v>0</v>
+      </c>
+      <c r="N92" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>507</v>
       </c>
@@ -4145,8 +4990,17 @@
       <c r="I93" s="5"/>
       <c r="J93" s="5"/>
       <c r="K93" s="5"/>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L93" t="b">
+        <v>0</v>
+      </c>
+      <c r="M93" t="b">
+        <v>0</v>
+      </c>
+      <c r="N93" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>508</v>
       </c>
@@ -4162,8 +5016,17 @@
         <v>1</v>
       </c>
       <c r="K94" s="5"/>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L94" t="b">
+        <v>0</v>
+      </c>
+      <c r="M94" t="b">
+        <v>0</v>
+      </c>
+      <c r="N94" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>471</v>
       </c>
@@ -4181,8 +5044,17 @@
       <c r="I95" s="5"/>
       <c r="J95" s="5"/>
       <c r="K95" s="5"/>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L95" t="b">
+        <v>1</v>
+      </c>
+      <c r="M95" t="b">
+        <v>0</v>
+      </c>
+      <c r="N95" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>509</v>
       </c>
@@ -4198,8 +5070,17 @@
       <c r="I96" s="5"/>
       <c r="J96" s="5"/>
       <c r="K96" s="5"/>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L96" t="b">
+        <v>0</v>
+      </c>
+      <c r="M96" t="b">
+        <v>0</v>
+      </c>
+      <c r="N96" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>510</v>
       </c>
@@ -4215,8 +5096,17 @@
       <c r="I97" s="5"/>
       <c r="J97" s="5"/>
       <c r="K97" s="5"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L97" t="b">
+        <v>0</v>
+      </c>
+      <c r="M97" t="b">
+        <v>0</v>
+      </c>
+      <c r="N97" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>511</v>
       </c>
@@ -4232,8 +5122,17 @@
         <v>1</v>
       </c>
       <c r="K98" s="5"/>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L98" t="b">
+        <v>0</v>
+      </c>
+      <c r="M98" t="b">
+        <v>0</v>
+      </c>
+      <c r="N98" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>475</v>
       </c>
@@ -4249,8 +5148,17 @@
       <c r="I99" s="5"/>
       <c r="J99" s="5"/>
       <c r="K99" s="5"/>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L99" t="b">
+        <v>0</v>
+      </c>
+      <c r="M99" t="b">
+        <v>0</v>
+      </c>
+      <c r="N99" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>512</v>
       </c>
@@ -4266,9 +5174,19 @@
       <c r="I100" s="5"/>
       <c r="J100" s="5"/>
       <c r="K100" s="5"/>
+      <c r="L100" t="b">
+        <v>0</v>
+      </c>
+      <c r="M100" t="b">
+        <v>0</v>
+      </c>
+      <c r="N100" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>